<commit_message>
fix: correct English event title
</commit_message>
<xml_diff>
--- a/outputs/019f8a8b-3448-7131-be8e-445e1a59680c/REFERENTI_080726_coerente_gruppi_iscrizioni_pace.xlsx
+++ b/outputs/019f8a8b-3448-7131-be8e-445e1a59680c/REFERENTI_080726_coerente_gruppi_iscrizioni_pace.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio1" sheetId="1" r:id="R08f826d62eb9426b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio2" sheetId="2" r:id="R4bbe29c79de14368"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referenti normalizzati" sheetId="3" r:id="R02a8bd1310f84ebe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo gruppi app" sheetId="4" r:id="R333d0f3e18a0455f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio1" sheetId="1" r:id="R0b1058ae8e114b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foglio2" sheetId="2" r:id="Rc257cfc6d35c47d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referenti normalizzati" sheetId="3" r:id="R400c7e75c0e0492a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo gruppi app" sheetId="4" r:id="R4d0247a82d614e04"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1382,7 +1382,7 @@
         <x:color rgb="FFA4231F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -1393,7 +1393,7 @@
         <x:color rgb="FF7A4A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1403,7 +1403,7 @@
         <x:color rgb="FF216E39"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEFE2"/>
         </x:patternFill>
       </x:fill>
@@ -1413,7 +1413,7 @@
         <x:color rgb="FF2458A6"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F0FE"/>
         </x:patternFill>
       </x:fill>
@@ -1424,7 +1424,7 @@
         <x:color rgb="FFA4231F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -1434,7 +1434,7 @@
         <x:color rgb="FF216E39"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEFE2"/>
         </x:patternFill>
       </x:fill>
@@ -4769,8 +4769,8 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R985a69c3d1dc4528"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="R91dcd28642ed4f56"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R227b1e5e4b414341"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="R13226afe01f24b74"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9731,7 +9731,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a7cd116bb48452d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ae07ab55f234bc6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9768,7 +9768,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>Evento corrente: UNHARMED AND DISARMING PEACE - PACE DISARMATA E DISARMANTE. Il conteggio dei referenti è calcolato dalla lista normalizzata tramite ID gruppo.</x:v>
+        <x:v>Evento corrente: UNARMED AND DISARMING PEACE - PACE DISARMATA E DISARMANTE. Il conteggio dei referenti è calcolato dalla lista normalizzata tramite ID gruppo.</x:v>
       </x:c>
       <x:c r="B2" s="9"/>
       <x:c r="C2" s="9"/>
@@ -12233,7 +12233,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea883f14154a4fd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafdfb577c79b4320"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>